<commit_message>
Mapping und durchschnittliches Gehalt aus BDB entfernt
</commit_message>
<xml_diff>
--- a/Speicherplatzberechnung_Bäckereikette.xlsx
+++ b/Speicherplatzberechnung_Bäckereikette.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alfa\Documents\Data Engineer\Projekt\BackZeit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{133998B3-4922-42DF-85AE-15F9301564D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC9D123-35EB-4D62-99C3-D9FCD167D2D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="3.NF" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="101">
   <si>
     <t>Filiale</t>
   </si>
@@ -107,9 +107,6 @@
   </si>
   <si>
     <t>Zahlart</t>
-  </si>
-  <si>
-    <t>durchschnittl. Umsatz</t>
   </si>
   <si>
     <t>Geschlecht</t>
@@ -920,7 +917,7 @@
         <v>21</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>21</v>
@@ -939,21 +936,19 @@
       <c r="B4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="4"/>
+      <c r="D4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>28</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>15</v>
@@ -962,78 +957,78 @@
         <v>15</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>32</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="I5" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="J5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" s="4" t="s">
         <v>35</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
       <c r="D7" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
@@ -1041,17 +1036,17 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -1059,17 +1054,17 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
@@ -1092,7 +1087,7 @@
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E11" s="4"/>
       <c r="G11" s="4"/>
@@ -1181,7 +1176,7 @@
         <v>11</v>
       </c>
       <c r="L20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
@@ -1207,7 +1202,7 @@
         <v>21</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>21</v>
@@ -1219,31 +1214,29 @@
         <v>13</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="4"/>
+      <c r="D22" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="E22" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H22" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>28</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>15</v>
@@ -1252,87 +1245,87 @@
         <v>15</v>
       </c>
       <c r="K22" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E23" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>32</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H23" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="I23" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="I23" s="4" t="s">
+      <c r="J23" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K23" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="J23" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="K23" s="4" t="s">
-        <v>36</v>
-      </c>
       <c r="L23" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H24" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="I24" s="4"/>
       <c r="J24" s="4"/>
       <c r="K24" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
@@ -1340,17 +1333,17 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="8"/>
       <c r="G26" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
@@ -1358,17 +1351,17 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
       <c r="D27" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
@@ -1378,7 +1371,7 @@
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
@@ -1391,7 +1384,7 @@
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E29" s="4"/>
       <c r="G29" s="4"/>
@@ -1425,7 +1418,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N126"/>
+  <dimension ref="A1:N125"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.140625" style="4" customWidth="1"/>
@@ -1512,7 +1505,7 @@
         <v>11</v>
       </c>
       <c r="L2" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -1538,7 +1531,7 @@
         <v>21</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>21</v>
@@ -1550,31 +1543,28 @@
         <v>13</v>
       </c>
       <c r="L3" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>28</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>15</v>
@@ -1583,115 +1573,115 @@
         <v>15</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>32</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>36</v>
-      </c>
       <c r="L5" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J7" s="4"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>46</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J8" s="4"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D9" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>50</v>
-      </c>
       <c r="G9" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J9" s="4"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10"/>
       <c r="D10" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F10" s="4"/>
       <c r="J10" s="4"/>
@@ -1699,7 +1689,7 @@
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11"/>
       <c r="D11" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
@@ -1710,46 +1700,46 @@
     </row>
     <row r="17" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="C17" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="D17" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="E17" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="F17" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="F17" s="13" t="s">
+      <c r="G17" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="G17" s="13" t="s">
+      <c r="H17" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="H17" s="13" t="s">
+      <c r="I17" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="I17" s="13" t="s">
+      <c r="J17" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="J17" s="13" t="s">
+      <c r="K17" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="K17" s="13" t="s">
+      <c r="L17" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="L17" s="13" t="s">
+      <c r="M17" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="M17" s="13" t="s">
+      <c r="N17" s="13" t="s">
         <v>73</v>
-      </c>
-      <c r="N17" s="13" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="15" x14ac:dyDescent="0.25">
@@ -1760,7 +1750,7 @@
         <v>11</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E18" s="19">
         <v>4</v>
@@ -1791,7 +1781,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D19" s="22">
         <v>50</v>
@@ -1818,10 +1808,10 @@
         <v>0</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D20" s="22"/>
       <c r="E20" s="19">
@@ -1846,10 +1836,10 @@
         <v>0</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D21" s="22">
         <v>7.2</v>
@@ -1874,10 +1864,10 @@
         <v>0</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D22" s="22">
         <v>7.2</v>
@@ -1902,10 +1892,10 @@
         <v>0</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D23" s="22">
         <v>7.2</v>
@@ -1929,10 +1919,10 @@
         <v>0</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D24" s="22">
         <v>7.2</v>
@@ -1957,10 +1947,10 @@
         <v>0</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D25" s="4">
         <v>7.2</v>
@@ -1988,13 +1978,13 @@
         <v>12</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E26" s="19">
         <v>8</v>
       </c>
       <c r="F26" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G26" s="20"/>
       <c r="H26" s="20"/>
@@ -2015,7 +2005,7 @@
         <v>11</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E27" s="24">
         <v>4</v>
@@ -2046,7 +2036,7 @@
         <v>23</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D28" s="4">
         <v>1</v>
@@ -2074,7 +2064,7 @@
         <v>13</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E29" s="25">
         <v>4</v>
@@ -2102,7 +2092,7 @@
         <v>13</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E30" s="24">
         <v>4</v>
@@ -2133,7 +2123,7 @@
         <v>14</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E31" s="25">
         <v>4</v>
@@ -2154,55 +2144,58 @@
     </row>
     <row r="32" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>24</v>
+        <v>3</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="D32" s="4">
-        <v>7.2</v>
-      </c>
-      <c r="E32" s="19">
-        <v>5</v>
-      </c>
-      <c r="F32" s="20"/>
+        <v>74</v>
+      </c>
+      <c r="E32" s="24">
+        <v>4</v>
+      </c>
+      <c r="F32" s="20">
+        <v>1</v>
+      </c>
       <c r="G32" s="20"/>
-      <c r="H32" s="20"/>
+      <c r="H32" s="20">
+        <v>1</v>
+      </c>
       <c r="I32" s="21"/>
       <c r="J32" s="21"/>
       <c r="K32" s="21"/>
-      <c r="M32" s="20"/>
+      <c r="L32" s="9">
+        <v>1</v>
+      </c>
+      <c r="M32" s="20">
+        <v>1</v>
+      </c>
       <c r="N32" s="21"/>
     </row>
     <row r="33" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>14</v>
+      <c r="B33" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="C33" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E33" s="24">
-        <v>4</v>
-      </c>
-      <c r="F33" s="20">
-        <v>1</v>
-      </c>
+      <c r="D33" s="22">
+        <v>50</v>
+      </c>
+      <c r="E33" s="19">
+        <f>2*D33+2</f>
+        <v>102</v>
+      </c>
+      <c r="F33" s="20"/>
       <c r="G33" s="20"/>
-      <c r="H33" s="20">
-        <v>1</v>
-      </c>
+      <c r="H33" s="20"/>
       <c r="I33" s="21"/>
       <c r="J33" s="21"/>
       <c r="K33" s="21"/>
-      <c r="L33" s="9">
-        <v>1</v>
-      </c>
       <c r="M33" s="20">
         <v>1</v>
       </c>
@@ -2213,17 +2206,16 @@
         <v>3</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="D34" s="22">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E34" s="19">
-        <f>2*D34+2</f>
-        <v>102</v>
+        <v>1</v>
       </c>
       <c r="F34" s="20"/>
       <c r="G34" s="20"/>
@@ -2231,9 +2223,7 @@
       <c r="I34" s="21"/>
       <c r="J34" s="21"/>
       <c r="K34" s="21"/>
-      <c r="M34" s="20">
-        <v>1</v>
-      </c>
+      <c r="M34" s="20"/>
       <c r="N34" s="21"/>
     </row>
     <row r="35" spans="1:14" ht="15" x14ac:dyDescent="0.25">
@@ -2241,16 +2231,16 @@
         <v>3</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>25</v>
+        <v>78</v>
       </c>
       <c r="C35" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D35" s="22">
-        <v>1</v>
+        <v>79</v>
+      </c>
+      <c r="D35" s="4">
+        <v>4.2</v>
       </c>
       <c r="E35" s="19">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F35" s="20"/>
       <c r="G35" s="20"/>
@@ -2258,7 +2248,9 @@
       <c r="I35" s="21"/>
       <c r="J35" s="21"/>
       <c r="K35" s="21"/>
-      <c r="M35" s="20"/>
+      <c r="M35" s="20">
+        <v>1</v>
+      </c>
       <c r="N35" s="21"/>
     </row>
     <row r="36" spans="1:14" ht="15" x14ac:dyDescent="0.25">
@@ -2266,16 +2258,13 @@
         <v>3</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="C36" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="D36" s="4">
-        <v>4.2</v>
+        <v>77</v>
       </c>
       <c r="E36" s="19">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F36" s="20"/>
       <c r="G36" s="20"/>
@@ -2283,9 +2272,7 @@
       <c r="I36" s="21"/>
       <c r="J36" s="21"/>
       <c r="K36" s="21"/>
-      <c r="M36" s="20">
-        <v>1</v>
-      </c>
+      <c r="M36" s="20"/>
       <c r="N36" s="21"/>
     </row>
     <row r="37" spans="1:14" ht="15" x14ac:dyDescent="0.25">
@@ -2293,13 +2280,16 @@
         <v>3</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>38</v>
+        <v>80</v>
       </c>
       <c r="C37" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
+      </c>
+      <c r="D37" s="4">
+        <v>4.2</v>
       </c>
       <c r="E37" s="19">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F37" s="20"/>
       <c r="G37" s="20"/>
@@ -2307,7 +2297,9 @@
       <c r="I37" s="21"/>
       <c r="J37" s="21"/>
       <c r="K37" s="21"/>
-      <c r="M37" s="20"/>
+      <c r="M37" s="20">
+        <v>1</v>
+      </c>
       <c r="N37" s="21"/>
     </row>
     <row r="38" spans="1:14" ht="15" x14ac:dyDescent="0.25">
@@ -2315,16 +2307,13 @@
         <v>3</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="D38" s="4">
-        <v>4.2</v>
+        <v>77</v>
       </c>
       <c r="E38" s="19">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F38" s="20"/>
       <c r="G38" s="20"/>
@@ -2342,13 +2331,17 @@
         <v>3</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C39" s="18" t="s">
-        <v>78</v>
+        <v>75</v>
+      </c>
+      <c r="D39" s="4">
+        <v>12</v>
       </c>
       <c r="E39" s="19">
-        <v>8</v>
+        <f>2*D39+2</f>
+        <v>26</v>
       </c>
       <c r="F39" s="20"/>
       <c r="G39" s="20"/>
@@ -2365,22 +2358,23 @@
       <c r="A40" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>49</v>
+      <c r="B40" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="C40" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="D40" s="4">
-        <v>12</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="D40" s="22"/>
       <c r="E40" s="19">
-        <f>2*D40+2</f>
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="F40" s="20"/>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
+      <c r="G40" s="20">
+        <v>1</v>
+      </c>
+      <c r="H40" s="20">
+        <v>1</v>
+      </c>
       <c r="I40" s="21"/>
       <c r="J40" s="21"/>
       <c r="K40" s="21"/>
@@ -2393,23 +2387,22 @@
       <c r="A41" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B41" s="5" t="s">
-        <v>52</v>
+      <c r="B41" s="4" t="s">
+        <v>50</v>
       </c>
       <c r="C41" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="D41" s="22"/>
+      <c r="D41" s="22">
+        <v>20</v>
+      </c>
       <c r="E41" s="19">
-        <v>4</v>
+        <f>2*D41+2</f>
+        <v>42</v>
       </c>
       <c r="F41" s="20"/>
-      <c r="G41" s="20">
-        <v>1</v>
-      </c>
-      <c r="H41" s="20">
-        <v>1</v>
-      </c>
+      <c r="G41" s="20"/>
+      <c r="H41" s="20"/>
       <c r="I41" s="21"/>
       <c r="J41" s="21"/>
       <c r="K41" s="21"/>
@@ -2420,59 +2413,58 @@
     </row>
     <row r="42" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>51</v>
+        <v>4</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="C42" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="D42" s="22">
-        <v>20</v>
-      </c>
-      <c r="E42" s="19">
-        <f>2*D42+2</f>
-        <v>42</v>
-      </c>
-      <c r="F42" s="20"/>
+        <v>74</v>
+      </c>
+      <c r="E42" s="24">
+        <v>4</v>
+      </c>
+      <c r="F42" s="20">
+        <v>1</v>
+      </c>
       <c r="G42" s="20"/>
-      <c r="H42" s="20"/>
+      <c r="H42" s="20">
+        <v>1</v>
+      </c>
       <c r="I42" s="21"/>
       <c r="J42" s="21"/>
       <c r="K42" s="21"/>
-      <c r="M42" s="20">
-        <v>1</v>
-      </c>
+      <c r="L42" s="9">
+        <v>1</v>
+      </c>
+      <c r="M42" s="20"/>
       <c r="N42" s="21"/>
     </row>
     <row r="43" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="2" t="s">
-        <v>15</v>
+      <c r="B43" s="4" t="s">
+        <v>20</v>
       </c>
       <c r="C43" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="E43" s="24">
-        <v>4</v>
-      </c>
-      <c r="F43" s="20">
-        <v>1</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="D43" s="4">
+        <v>4.2</v>
+      </c>
+      <c r="E43" s="19">
+        <v>5</v>
+      </c>
+      <c r="F43" s="20"/>
       <c r="G43" s="20"/>
-      <c r="H43" s="20">
-        <v>1</v>
-      </c>
+      <c r="H43" s="20"/>
       <c r="I43" s="21"/>
       <c r="J43" s="21"/>
       <c r="K43" s="21"/>
-      <c r="L43" s="9">
-        <v>1</v>
-      </c>
-      <c r="M43" s="20"/>
+      <c r="M43" s="20">
+        <v>1</v>
+      </c>
       <c r="N43" s="21"/>
     </row>
     <row r="44" spans="1:14" ht="15" x14ac:dyDescent="0.25">
@@ -2480,12 +2472,12 @@
         <v>4</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C44" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="D44" s="4">
+        <v>79</v>
+      </c>
+      <c r="D44" s="22">
         <v>4.2</v>
       </c>
       <c r="E44" s="19">
@@ -2497,6 +2489,7 @@
       <c r="I44" s="21"/>
       <c r="J44" s="21"/>
       <c r="K44" s="21"/>
+      <c r="L44" s="20"/>
       <c r="M44" s="20">
         <v>1</v>
       </c>
@@ -2507,16 +2500,17 @@
         <v>4</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C45" s="18" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D45" s="22">
-        <v>4.2</v>
+        <v>50</v>
       </c>
       <c r="E45" s="19">
-        <v>5</v>
+        <f>2*D45+2</f>
+        <v>102</v>
       </c>
       <c r="F45" s="20"/>
       <c r="G45" s="20"/>
@@ -2524,7 +2518,9 @@
       <c r="I45" s="21"/>
       <c r="J45" s="21"/>
       <c r="K45" s="21"/>
-      <c r="L45" s="20"/>
+      <c r="L45" s="20">
+        <v>1</v>
+      </c>
       <c r="M45" s="20">
         <v>1</v>
       </c>
@@ -2534,28 +2530,26 @@
       <c r="A46" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B46" s="4" t="s">
-        <v>32</v>
+      <c r="B46" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="C46" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="D46" s="22">
-        <v>50</v>
-      </c>
-      <c r="E46" s="19">
-        <f>2*D46+2</f>
-        <v>102</v>
+        <v>74</v>
+      </c>
+      <c r="E46" s="25">
+        <v>4</v>
       </c>
       <c r="F46" s="20"/>
-      <c r="G46" s="20"/>
-      <c r="H46" s="20"/>
+      <c r="G46" s="20">
+        <v>1</v>
+      </c>
+      <c r="H46" s="20">
+        <v>1</v>
+      </c>
       <c r="I46" s="21"/>
       <c r="J46" s="21"/>
       <c r="K46" s="21"/>
-      <c r="L46" s="20">
-        <v>1</v>
-      </c>
+      <c r="L46" s="20"/>
       <c r="M46" s="20">
         <v>1</v>
       </c>
@@ -2563,28 +2557,30 @@
     </row>
     <row r="47" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="B47" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C47" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E47" s="25">
         <v>4</v>
       </c>
-      <c r="F47" s="20"/>
-      <c r="G47" s="20">
-        <v>1</v>
-      </c>
+      <c r="F47" s="20">
+        <v>1</v>
+      </c>
+      <c r="G47" s="20"/>
       <c r="H47" s="20">
         <v>1</v>
       </c>
       <c r="I47" s="21"/>
       <c r="J47" s="21"/>
       <c r="K47" s="21"/>
-      <c r="L47" s="20"/>
+      <c r="L47" s="20">
+        <v>1</v>
+      </c>
       <c r="M47" s="20">
         <v>1</v>
       </c>
@@ -2594,22 +2590,22 @@
       <c r="A48" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>16</v>
+      <c r="B48" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="C48" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E48" s="25">
-        <v>4</v>
-      </c>
-      <c r="F48" s="20">
-        <v>1</v>
-      </c>
+      <c r="D48" s="22">
+        <v>50</v>
+      </c>
+      <c r="E48" s="19">
+        <f>2*D48+2</f>
+        <v>102</v>
+      </c>
+      <c r="F48" s="20"/>
       <c r="G48" s="20"/>
-      <c r="H48" s="20">
-        <v>1</v>
-      </c>
+      <c r="H48" s="20"/>
       <c r="I48" s="21"/>
       <c r="J48" s="21"/>
       <c r="K48" s="21"/>
@@ -2623,30 +2619,30 @@
     </row>
     <row r="49" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="23" t="s">
-        <v>5</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>19</v>
+        <v>6</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="C49" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="D49" s="22">
-        <v>50</v>
-      </c>
-      <c r="E49" s="19">
-        <f>2*D49+2</f>
-        <v>102</v>
-      </c>
-      <c r="F49" s="20"/>
-      <c r="G49" s="20"/>
-      <c r="H49" s="20"/>
+        <v>74</v>
+      </c>
+      <c r="E49" s="25">
+        <v>4</v>
+      </c>
+      <c r="F49" s="20">
+        <v>1</v>
+      </c>
+      <c r="G49" s="20">
+        <v>1</v>
+      </c>
+      <c r="H49" s="20">
+        <v>1</v>
+      </c>
       <c r="I49" s="21"/>
       <c r="J49" s="21"/>
       <c r="K49" s="21"/>
-      <c r="L49" s="20">
-        <v>1</v>
-      </c>
+      <c r="L49" s="20"/>
       <c r="M49" s="20">
         <v>1</v>
       </c>
@@ -2657,20 +2653,19 @@
         <v>6</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C50" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="E50" s="25">
-        <v>4</v>
+        <v>81</v>
+      </c>
+      <c r="D50" s="22"/>
+      <c r="E50" s="19">
+        <v>2</v>
       </c>
       <c r="F50" s="20">
         <v>1</v>
       </c>
-      <c r="G50" s="20">
-        <v>1</v>
-      </c>
+      <c r="G50" s="20"/>
       <c r="H50" s="20">
         <v>1</v>
       </c>
@@ -2687,23 +2682,21 @@
       <c r="A51" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>21</v>
+      <c r="B51" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="C51" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="D51" s="22"/>
+        <v>79</v>
+      </c>
+      <c r="D51" s="22">
+        <v>4.2</v>
+      </c>
       <c r="E51" s="19">
-        <v>2</v>
-      </c>
-      <c r="F51" s="20">
-        <v>1</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="F51" s="20"/>
       <c r="G51" s="20"/>
-      <c r="H51" s="20">
-        <v>1</v>
-      </c>
+      <c r="H51" s="20"/>
       <c r="I51" s="21"/>
       <c r="J51" s="21"/>
       <c r="K51" s="21"/>
@@ -2718,16 +2711,14 @@
         <v>6</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C52" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="D52" s="22">
-        <v>4.2</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="D52" s="22"/>
       <c r="E52" s="19">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F52" s="20"/>
       <c r="G52" s="20"/>
@@ -2736,9 +2727,7 @@
       <c r="J52" s="21"/>
       <c r="K52" s="21"/>
       <c r="L52" s="20"/>
-      <c r="M52" s="20">
-        <v>1</v>
-      </c>
+      <c r="M52" s="20"/>
       <c r="N52" s="21"/>
     </row>
     <row r="53" spans="1:14" ht="15" x14ac:dyDescent="0.25">
@@ -2746,10 +2735,10 @@
         <v>6</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C53" s="18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D53" s="22"/>
       <c r="E53" s="19">
@@ -2770,14 +2759,16 @@
         <v>6</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="D54" s="22"/>
+        <v>79</v>
+      </c>
+      <c r="D54" s="22">
+        <v>4.2</v>
+      </c>
       <c r="E54" s="19">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F54" s="20"/>
       <c r="G54" s="20"/>
@@ -2786,7 +2777,9 @@
       <c r="J54" s="21"/>
       <c r="K54" s="21"/>
       <c r="L54" s="20"/>
-      <c r="M54" s="20"/>
+      <c r="M54" s="20">
+        <v>1</v>
+      </c>
       <c r="N54" s="21"/>
     </row>
     <row r="55" spans="1:14" ht="15" x14ac:dyDescent="0.25">
@@ -2794,16 +2787,17 @@
         <v>6</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D55" s="22">
-        <v>4.2</v>
+        <v>50</v>
       </c>
       <c r="E55" s="19">
-        <v>5</v>
+        <f>2*D55+2</f>
+        <v>102</v>
       </c>
       <c r="F55" s="20"/>
       <c r="G55" s="20"/>
@@ -2822,17 +2816,14 @@
         <v>6</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C56" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="D56" s="22">
-        <v>50</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="D56" s="22"/>
       <c r="E56" s="19">
-        <f>2*D56+2</f>
-        <v>102</v>
+        <v>1</v>
       </c>
       <c r="F56" s="20"/>
       <c r="G56" s="20"/>
@@ -2841,61 +2832,63 @@
       <c r="J56" s="21"/>
       <c r="K56" s="21"/>
       <c r="L56" s="20"/>
-      <c r="M56" s="20">
-        <v>1</v>
-      </c>
+      <c r="M56" s="20"/>
       <c r="N56" s="21"/>
     </row>
     <row r="57" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>50</v>
+        <v>7</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="C57" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="D57" s="22"/>
-      <c r="E57" s="19">
-        <v>1</v>
-      </c>
-      <c r="F57" s="20"/>
+        <v>74</v>
+      </c>
+      <c r="E57" s="25">
+        <v>4</v>
+      </c>
+      <c r="F57" s="20">
+        <v>1</v>
+      </c>
       <c r="G57" s="20"/>
-      <c r="H57" s="20"/>
+      <c r="H57" s="20">
+        <v>1</v>
+      </c>
       <c r="I57" s="21"/>
       <c r="J57" s="21"/>
       <c r="K57" s="21"/>
-      <c r="L57" s="20"/>
-      <c r="M57" s="20"/>
+      <c r="L57" s="20">
+        <v>1</v>
+      </c>
+      <c r="M57" s="20">
+        <v>1</v>
+      </c>
       <c r="N57" s="21"/>
     </row>
     <row r="58" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>17</v>
+      <c r="B58" s="4" t="s">
+        <v>100</v>
       </c>
       <c r="C58" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="E58" s="25">
-        <v>4</v>
-      </c>
-      <c r="F58" s="20">
-        <v>1</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="D58" s="22">
+        <v>4.2</v>
+      </c>
+      <c r="E58" s="19">
+        <v>5</v>
+      </c>
+      <c r="F58" s="20"/>
       <c r="G58" s="20"/>
-      <c r="H58" s="20">
-        <v>1</v>
-      </c>
+      <c r="H58" s="20"/>
       <c r="I58" s="21"/>
       <c r="J58" s="21"/>
       <c r="K58" s="21"/>
-      <c r="L58" s="20">
-        <v>1</v>
-      </c>
+      <c r="L58" s="20"/>
       <c r="M58" s="20">
         <v>1</v>
       </c>
@@ -2906,17 +2899,13 @@
         <v>7</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>101</v>
+        <v>27</v>
       </c>
       <c r="C59" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="D59" s="22">
-        <v>4.2</v>
-      </c>
-      <c r="E59" s="19">
-        <v>5</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D59" s="22"/>
+      <c r="E59" s="19"/>
       <c r="F59" s="20"/>
       <c r="G59" s="20"/>
       <c r="H59" s="20"/>
@@ -2924,9 +2913,7 @@
       <c r="J59" s="21"/>
       <c r="K59" s="21"/>
       <c r="L59" s="20"/>
-      <c r="M59" s="20">
-        <v>1</v>
-      </c>
+      <c r="M59" s="20"/>
       <c r="N59" s="21"/>
     </row>
     <row r="60" spans="1:14" ht="15" x14ac:dyDescent="0.25">
@@ -2934,13 +2921,17 @@
         <v>7</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="C60" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="D60" s="22"/>
-      <c r="E60" s="19"/>
+        <v>76</v>
+      </c>
+      <c r="D60" s="22">
+        <v>7.2</v>
+      </c>
+      <c r="E60" s="19">
+        <v>5</v>
+      </c>
       <c r="F60" s="20"/>
       <c r="G60" s="20"/>
       <c r="H60" s="20"/>
@@ -2948,7 +2939,9 @@
       <c r="J60" s="21"/>
       <c r="K60" s="21"/>
       <c r="L60" s="20"/>
-      <c r="M60" s="20"/>
+      <c r="M60" s="20">
+        <v>1</v>
+      </c>
       <c r="N60" s="21"/>
     </row>
     <row r="61" spans="1:14" ht="15" x14ac:dyDescent="0.25">
@@ -2956,16 +2949,17 @@
         <v>7</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="C61" s="18" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D61" s="22">
-        <v>7.2</v>
+        <v>50</v>
       </c>
       <c r="E61" s="19">
-        <v>5</v>
+        <f>2*D642+2</f>
+        <v>2</v>
       </c>
       <c r="F61" s="20"/>
       <c r="G61" s="20"/>
@@ -2973,7 +2967,9 @@
       <c r="I61" s="21"/>
       <c r="J61" s="21"/>
       <c r="K61" s="21"/>
-      <c r="L61" s="20"/>
+      <c r="L61" s="20">
+        <v>1</v>
+      </c>
       <c r="M61" s="20">
         <v>1</v>
       </c>
@@ -2981,30 +2977,30 @@
     </row>
     <row r="62" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>40</v>
+        <v>8</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="C62" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="D62" s="22">
-        <v>50</v>
-      </c>
-      <c r="E62" s="19">
-        <f>2*D643+2</f>
-        <v>2</v>
-      </c>
-      <c r="F62" s="20"/>
-      <c r="G62" s="20"/>
-      <c r="H62" s="20"/>
+        <v>74</v>
+      </c>
+      <c r="E62" s="25">
+        <v>4</v>
+      </c>
+      <c r="F62" s="20">
+        <v>1</v>
+      </c>
+      <c r="G62" s="20">
+        <v>1</v>
+      </c>
+      <c r="H62" s="20">
+        <v>1</v>
+      </c>
       <c r="I62" s="21"/>
       <c r="J62" s="21"/>
       <c r="K62" s="21"/>
-      <c r="L62" s="20">
-        <v>1</v>
-      </c>
+      <c r="L62" s="20"/>
       <c r="M62" s="20">
         <v>1</v>
       </c>
@@ -3015,13 +3011,13 @@
         <v>8</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C63" s="18" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="E63" s="25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F63" s="20">
         <v>1</v>
@@ -3046,13 +3042,13 @@
         <v>8</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C64" s="18" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="E64" s="25">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F64" s="20">
         <v>1</v>
@@ -3076,24 +3072,18 @@
       <c r="A65" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B65" s="3" t="s">
-        <v>15</v>
+      <c r="B65" s="4" t="s">
+        <v>34</v>
       </c>
       <c r="C65" s="18" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="E65" s="25">
-        <v>4</v>
-      </c>
-      <c r="F65" s="20">
-        <v>1</v>
-      </c>
-      <c r="G65" s="20">
-        <v>1</v>
-      </c>
-      <c r="H65" s="20">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F65" s="20"/>
+      <c r="G65" s="20"/>
+      <c r="H65" s="20"/>
       <c r="I65" s="21"/>
       <c r="J65" s="21"/>
       <c r="K65" s="21"/>
@@ -3105,20 +3095,26 @@
     </row>
     <row r="66" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="B66" s="4" t="s">
-        <v>35</v>
+        <v>9</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="C66" s="18" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="E66" s="25">
-        <v>2</v>
-      </c>
-      <c r="F66" s="20"/>
-      <c r="G66" s="20"/>
-      <c r="H66" s="20"/>
+        <v>4</v>
+      </c>
+      <c r="F66" s="20">
+        <v>1</v>
+      </c>
+      <c r="G66" s="20">
+        <v>1</v>
+      </c>
+      <c r="H66" s="20">
+        <v>1</v>
+      </c>
       <c r="I66" s="21"/>
       <c r="J66" s="21"/>
       <c r="K66" s="21"/>
@@ -3133,13 +3129,14 @@
         <v>9</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C67" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="E67" s="25">
-        <v>4</v>
+        <v>77</v>
+      </c>
+      <c r="D67" s="22"/>
+      <c r="E67" s="19">
+        <v>8</v>
       </c>
       <c r="F67" s="20">
         <v>1</v>
@@ -3164,14 +3161,14 @@
         <v>9</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C68" s="18" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D68" s="22"/>
       <c r="E68" s="19">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F68" s="20">
         <v>1</v>
@@ -3195,25 +3192,21 @@
       <c r="A69" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="B69" s="3" t="s">
-        <v>15</v>
+      <c r="B69" s="4" t="s">
+        <v>34</v>
       </c>
       <c r="C69" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="D69" s="22"/>
+        <v>83</v>
+      </c>
+      <c r="D69" s="22">
+        <v>5.2</v>
+      </c>
       <c r="E69" s="19">
-        <v>4</v>
-      </c>
-      <c r="F69" s="20">
-        <v>1</v>
-      </c>
-      <c r="G69" s="20">
-        <v>1</v>
-      </c>
-      <c r="H69" s="20">
-        <v>1</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="F69" s="20"/>
+      <c r="G69" s="20"/>
+      <c r="H69" s="20"/>
       <c r="I69" s="21"/>
       <c r="J69" s="21"/>
       <c r="K69" s="21"/>
@@ -3225,23 +3218,27 @@
     </row>
     <row r="70" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A70" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="B70" s="4" t="s">
-        <v>35</v>
+        <v>10</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="C70" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="D70" s="22">
-        <v>5.2</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="D70" s="22"/>
       <c r="E70" s="19">
-        <v>5</v>
-      </c>
-      <c r="F70" s="20"/>
-      <c r="G70" s="20"/>
-      <c r="H70" s="20"/>
+        <v>4</v>
+      </c>
+      <c r="F70" s="20">
+        <v>1</v>
+      </c>
+      <c r="G70" s="20">
+        <v>1</v>
+      </c>
+      <c r="H70" s="20">
+        <v>1</v>
+      </c>
       <c r="I70" s="21"/>
       <c r="J70" s="21"/>
       <c r="K70" s="21"/>
@@ -3256,10 +3253,10 @@
         <v>10</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C71" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D71" s="22"/>
       <c r="E71" s="19">
@@ -3287,25 +3284,19 @@
       <c r="A72" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="B72" s="3" t="s">
-        <v>13</v>
+      <c r="B72" s="4" t="s">
+        <v>28</v>
       </c>
       <c r="C72" s="18" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="D72" s="22"/>
       <c r="E72" s="19">
-        <v>4</v>
-      </c>
-      <c r="F72" s="20">
-        <v>1</v>
-      </c>
-      <c r="G72" s="20">
-        <v>1</v>
-      </c>
-      <c r="H72" s="20">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="F72" s="20"/>
+      <c r="G72" s="20"/>
+      <c r="H72" s="20"/>
       <c r="I72" s="21"/>
       <c r="J72" s="21"/>
       <c r="K72" s="21"/>
@@ -3320,14 +3311,14 @@
         <v>10</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C73" s="18" t="s">
         <v>85</v>
       </c>
       <c r="D73" s="22"/>
       <c r="E73" s="19">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F73" s="20"/>
       <c r="G73" s="20"/>
@@ -3346,10 +3337,10 @@
         <v>10</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C74" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D74" s="22"/>
       <c r="E74" s="19">
@@ -3369,25 +3360,31 @@
     </row>
     <row r="75" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A75" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="B75" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C75" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="D75" s="22"/>
-      <c r="E75" s="19">
-        <v>5</v>
-      </c>
-      <c r="F75" s="20"/>
+        <v>22</v>
+      </c>
+      <c r="B75" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C75" t="s">
+        <v>74</v>
+      </c>
+      <c r="D75"/>
+      <c r="E75" s="26">
+        <v>4</v>
+      </c>
+      <c r="F75" s="20">
+        <v>1</v>
+      </c>
       <c r="G75" s="20"/>
-      <c r="H75" s="20"/>
+      <c r="H75" s="20">
+        <v>1</v>
+      </c>
       <c r="I75" s="21"/>
       <c r="J75" s="21"/>
       <c r="K75" s="21"/>
-      <c r="L75" s="20"/>
+      <c r="L75" s="20">
+        <v>1</v>
+      </c>
       <c r="M75" s="20">
         <v>1</v>
       </c>
@@ -3397,29 +3394,26 @@
       <c r="A76" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="B76" s="12" t="s">
+      <c r="B76" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C76" t="s">
+      <c r="C76" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="D76"/>
-      <c r="E76" s="26">
-        <v>4</v>
-      </c>
-      <c r="F76" s="20">
-        <v>1</v>
-      </c>
+      <c r="D76" s="22">
+        <v>50</v>
+      </c>
+      <c r="E76" s="19">
+        <f>2*D76+2</f>
+        <v>102</v>
+      </c>
+      <c r="F76" s="20"/>
       <c r="G76" s="20"/>
-      <c r="H76" s="20">
-        <v>1</v>
-      </c>
+      <c r="H76" s="20"/>
       <c r="I76" s="21"/>
       <c r="J76" s="21"/>
       <c r="K76" s="21"/>
-      <c r="L76" s="20">
-        <v>1</v>
-      </c>
+      <c r="L76" s="20"/>
       <c r="M76" s="20">
         <v>1</v>
       </c>
@@ -3433,14 +3427,13 @@
         <v>53</v>
       </c>
       <c r="C77" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="D77" s="22">
-        <v>50</v>
+        <v>86</v>
+      </c>
+      <c r="D77" s="4">
+        <v>5</v>
       </c>
       <c r="E77" s="19">
-        <f>2*D77+2</f>
-        <v>102</v>
+        <v>7</v>
       </c>
       <c r="F77" s="20"/>
       <c r="G77" s="20"/>
@@ -3462,13 +3455,14 @@
         <v>54</v>
       </c>
       <c r="C78" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="D78" s="4">
-        <v>5</v>
+        <v>75</v>
+      </c>
+      <c r="D78" s="22">
+        <v>2</v>
       </c>
       <c r="E78" s="19">
-        <v>7</v>
+        <f>2*D78+2</f>
+        <v>6</v>
       </c>
       <c r="F78" s="20"/>
       <c r="G78" s="20"/>
@@ -3490,14 +3484,14 @@
         <v>55</v>
       </c>
       <c r="C79" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="D79" s="22">
-        <v>2</v>
+        <v>75</v>
+      </c>
+      <c r="D79" s="4">
+        <v>7</v>
       </c>
       <c r="E79" s="19">
         <f>2*D79+2</f>
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F79" s="20"/>
       <c r="G79" s="20"/>
@@ -3511,47 +3505,36 @@
       </c>
       <c r="N79" s="21"/>
     </row>
-    <row r="80" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A80" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C80" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="D80" s="4">
-        <v>7</v>
-      </c>
-      <c r="E80" s="19">
-        <f>2*D80+2</f>
-        <v>16</v>
-      </c>
-      <c r="F80" s="20"/>
-      <c r="G80" s="20"/>
-      <c r="H80" s="20"/>
+    <row r="80" spans="1:14" ht="18" x14ac:dyDescent="0.25">
+      <c r="A80" s="42" t="s">
+        <v>87</v>
+      </c>
+      <c r="B80" s="42"/>
+      <c r="C80" s="27"/>
+      <c r="D80" s="21"/>
+      <c r="E80" s="21"/>
+      <c r="F80" s="21"/>
+      <c r="G80" s="21"/>
+      <c r="H80" s="21"/>
       <c r="I80" s="21"/>
       <c r="J80" s="21"/>
       <c r="K80" s="21"/>
       <c r="L80" s="20"/>
-      <c r="M80" s="20">
-        <v>1</v>
-      </c>
+      <c r="M80" s="20"/>
       <c r="N80" s="21"/>
     </row>
-    <row r="81" spans="1:14" ht="18" x14ac:dyDescent="0.25">
-      <c r="A81" s="42" t="s">
+    <row r="81" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="A81" s="43" t="s">
         <v>88</v>
       </c>
-      <c r="B81" s="42"/>
-      <c r="C81" s="27"/>
-      <c r="D81" s="21"/>
-      <c r="E81" s="21"/>
-      <c r="F81" s="21"/>
-      <c r="G81" s="21"/>
-      <c r="H81" s="21"/>
-      <c r="I81" s="21"/>
+      <c r="B81" s="43"/>
+      <c r="C81" s="43"/>
+      <c r="D81" s="43"/>
+      <c r="E81" s="43"/>
+      <c r="F81" s="43"/>
+      <c r="G81" s="28"/>
+      <c r="H81" s="28"/>
+      <c r="I81" s="28"/>
       <c r="J81" s="21"/>
       <c r="K81" s="21"/>
       <c r="L81" s="20"/>
@@ -3559,68 +3542,90 @@
       <c r="N81" s="21"/>
     </row>
     <row r="82" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A82" s="43" t="s">
+      <c r="A82" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="B82" s="43"/>
-      <c r="C82" s="43"/>
-      <c r="D82" s="43"/>
-      <c r="E82" s="43"/>
-      <c r="F82" s="43"/>
-      <c r="G82" s="28"/>
-      <c r="H82" s="28"/>
-      <c r="I82" s="28"/>
+      <c r="B82" s="44"/>
+      <c r="C82" s="29"/>
+      <c r="D82" s="21"/>
+      <c r="E82" s="21"/>
+      <c r="F82" s="21"/>
+      <c r="G82" s="21"/>
+      <c r="H82" s="21"/>
+      <c r="I82" s="21"/>
       <c r="J82" s="21"/>
       <c r="K82" s="21"/>
       <c r="L82" s="20"/>
       <c r="M82" s="20"/>
       <c r="N82" s="21"/>
     </row>
-    <row r="83" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A83" s="44" t="s">
+    <row r="83" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A83" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="B83" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="B83" s="44"/>
-      <c r="C83" s="29"/>
-      <c r="D83" s="21"/>
-      <c r="E83" s="21"/>
-      <c r="F83" s="21"/>
-      <c r="G83" s="21"/>
-      <c r="H83" s="21"/>
-      <c r="I83" s="21"/>
+      <c r="C83" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="D83" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="E83" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="F83" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="G83" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="H83" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="I83" s="32" t="s">
+        <v>97</v>
+      </c>
       <c r="J83" s="21"/>
       <c r="K83" s="21"/>
       <c r="L83" s="20"/>
       <c r="M83" s="20"/>
       <c r="N83" s="21"/>
     </row>
-    <row r="84" spans="1:14" ht="60" x14ac:dyDescent="0.25">
-      <c r="A84" s="30" t="s">
-        <v>61</v>
-      </c>
-      <c r="B84" s="31" t="s">
-        <v>91</v>
-      </c>
-      <c r="C84" s="31" t="s">
-        <v>92</v>
-      </c>
-      <c r="D84" s="32" t="s">
-        <v>93</v>
-      </c>
-      <c r="E84" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="F84" s="32" t="s">
-        <v>95</v>
-      </c>
-      <c r="G84" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="H84" s="32" t="s">
-        <v>97</v>
-      </c>
-      <c r="I84" s="32" t="s">
-        <v>98</v>
+    <row r="84" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="A84" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B84" s="4">
+        <v>50</v>
+      </c>
+      <c r="C84" s="4">
+        <v>5</v>
+      </c>
+      <c r="D84" s="19">
+        <f t="shared" ref="D84:D95" si="0">B84+10*C84</f>
+        <v>100</v>
+      </c>
+      <c r="E84" s="19">
+        <f>SUM(E18:E25)</f>
+        <v>135</v>
+      </c>
+      <c r="F84" s="19">
+        <f t="shared" ref="F84:F95" si="1">D84*E84</f>
+        <v>13500</v>
+      </c>
+      <c r="G84" s="34">
+        <f t="shared" ref="G84:I95" si="2">F84/1024</f>
+        <v>13.18359375</v>
+      </c>
+      <c r="H84" s="34">
+        <f t="shared" si="2"/>
+        <v>1.2874603271484375E-2</v>
+      </c>
+      <c r="I84" s="19">
+        <f t="shared" si="2"/>
+        <v>1.257285475730896E-5</v>
       </c>
       <c r="J84" s="21"/>
       <c r="K84" s="21"/>
@@ -3629,38 +3634,38 @@
       <c r="N84" s="21"/>
     </row>
     <row r="85" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A85" s="33" t="s">
-        <v>0</v>
-      </c>
-      <c r="B85" s="4">
-        <v>50</v>
-      </c>
-      <c r="C85" s="4">
-        <v>5</v>
+      <c r="A85" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B85" s="36">
+        <v>10000000</v>
+      </c>
+      <c r="C85" s="36">
+        <v>11000000</v>
       </c>
       <c r="D85" s="19">
-        <f t="shared" ref="D85:D96" si="0">B85+10*C85</f>
-        <v>100</v>
+        <f t="shared" si="0"/>
+        <v>120000000</v>
       </c>
       <c r="E85" s="19">
-        <f>SUM(E18:E25)</f>
-        <v>135</v>
+        <f>SUM(E26:E29)</f>
+        <v>17</v>
       </c>
       <c r="F85" s="19">
-        <f t="shared" ref="F85:F96" si="1">D85*E85</f>
-        <v>13500</v>
+        <f t="shared" si="1"/>
+        <v>2040000000</v>
       </c>
       <c r="G85" s="34">
-        <f t="shared" ref="G85:I96" si="2">F85/1024</f>
-        <v>13.18359375</v>
+        <f t="shared" si="2"/>
+        <v>1992187.5</v>
       </c>
       <c r="H85" s="34">
         <f t="shared" si="2"/>
-        <v>1.2874603271484375E-2</v>
+        <v>1945.49560546875</v>
       </c>
       <c r="I85" s="19">
         <f t="shared" si="2"/>
-        <v>1.257285475730896E-5</v>
+        <v>1.8998980522155762</v>
       </c>
       <c r="J85" s="21"/>
       <c r="K85" s="21"/>
@@ -3670,37 +3675,37 @@
     </row>
     <row r="86" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A86" s="35" t="s">
-        <v>1</v>
-      </c>
-      <c r="B86" s="36">
-        <v>10000000</v>
-      </c>
-      <c r="C86" s="36">
-        <v>11000000</v>
+        <v>2</v>
+      </c>
+      <c r="B86" s="4">
+        <v>150</v>
+      </c>
+      <c r="C86" s="4">
+        <v>30</v>
       </c>
       <c r="D86" s="19">
         <f t="shared" si="0"/>
-        <v>120000000</v>
+        <v>450</v>
       </c>
       <c r="E86" s="19">
-        <f>SUM(E26:E29)</f>
-        <v>17</v>
+        <f>SUM(E30:E31)</f>
+        <v>8</v>
       </c>
       <c r="F86" s="19">
         <f t="shared" si="1"/>
-        <v>2040000000</v>
+        <v>3600</v>
       </c>
       <c r="G86" s="34">
         <f t="shared" si="2"/>
-        <v>1992187.5</v>
+        <v>3.515625</v>
       </c>
       <c r="H86" s="34">
         <f t="shared" si="2"/>
-        <v>1945.49560546875</v>
+        <v>3.4332275390625E-3</v>
       </c>
       <c r="I86" s="19">
         <f t="shared" si="2"/>
-        <v>1.8998980522155762</v>
+        <v>3.3527612686157227E-6</v>
       </c>
       <c r="J86" s="21"/>
       <c r="K86" s="21"/>
@@ -3710,37 +3715,37 @@
     </row>
     <row r="87" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A87" s="35" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B87" s="4">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C87" s="4">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D87" s="19">
         <f t="shared" si="0"/>
-        <v>450</v>
+        <v>540</v>
       </c>
       <c r="E87" s="19">
-        <f>SUM(E30:E32)</f>
-        <v>13</v>
+        <f>SUM(E32:E41)</f>
+        <v>205</v>
       </c>
       <c r="F87" s="19">
         <f t="shared" si="1"/>
-        <v>5850</v>
+        <v>110700</v>
       </c>
       <c r="G87" s="34">
         <f t="shared" si="2"/>
-        <v>5.712890625</v>
+        <v>108.10546875</v>
       </c>
       <c r="H87" s="34">
         <f t="shared" si="2"/>
-        <v>5.5789947509765625E-3</v>
+        <v>0.10557174682617188</v>
       </c>
       <c r="I87" s="19">
         <f t="shared" si="2"/>
-        <v>5.4482370615005493E-6</v>
+        <v>1.0309740900993347E-4</v>
       </c>
       <c r="J87" s="21"/>
       <c r="K87" s="21"/>
@@ -3750,37 +3755,37 @@
     </row>
     <row r="88" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A88" s="35" t="s">
-        <v>3</v>
-      </c>
-      <c r="B88" s="4">
-        <v>200</v>
-      </c>
-      <c r="C88" s="4">
-        <v>34</v>
+        <v>4</v>
+      </c>
+      <c r="B88" s="21">
+        <v>50</v>
+      </c>
+      <c r="C88" s="21">
+        <v>5</v>
       </c>
       <c r="D88" s="19">
         <f t="shared" si="0"/>
-        <v>540</v>
+        <v>100</v>
       </c>
       <c r="E88" s="19">
-        <f>SUM(E33:E42)</f>
-        <v>205</v>
+        <f>SUM(E42:E46)</f>
+        <v>120</v>
       </c>
       <c r="F88" s="19">
         <f t="shared" si="1"/>
-        <v>110700</v>
+        <v>12000</v>
       </c>
       <c r="G88" s="34">
         <f t="shared" si="2"/>
-        <v>108.10546875</v>
+        <v>11.71875</v>
       </c>
       <c r="H88" s="34">
         <f t="shared" si="2"/>
-        <v>0.10557174682617188</v>
+        <v>1.1444091796875E-2</v>
       </c>
       <c r="I88" s="19">
         <f t="shared" si="2"/>
-        <v>1.0309740900993347E-4</v>
+        <v>1.1175870895385742E-5</v>
       </c>
       <c r="J88" s="21"/>
       <c r="K88" s="21"/>
@@ -3789,38 +3794,38 @@
       <c r="N88" s="21"/>
     </row>
     <row r="89" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A89" s="35" t="s">
-        <v>4</v>
-      </c>
-      <c r="B89" s="21">
-        <v>50</v>
-      </c>
-      <c r="C89" s="21">
+      <c r="A89" s="37" t="s">
         <v>5</v>
+      </c>
+      <c r="B89" s="4">
+        <v>6</v>
+      </c>
+      <c r="C89" s="4">
+        <v>0</v>
       </c>
       <c r="D89" s="19">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="E89" s="19">
-        <f>SUM(E43:E47)</f>
-        <v>120</v>
+        <f>SUM(E47:E48)</f>
+        <v>106</v>
       </c>
       <c r="F89" s="19">
         <f t="shared" si="1"/>
-        <v>12000</v>
+        <v>636</v>
       </c>
       <c r="G89" s="34">
         <f t="shared" si="2"/>
-        <v>11.71875</v>
+        <v>0.62109375</v>
       </c>
       <c r="H89" s="34">
         <f t="shared" si="2"/>
-        <v>1.1444091796875E-2</v>
+        <v>6.06536865234375E-4</v>
       </c>
       <c r="I89" s="19">
         <f t="shared" si="2"/>
-        <v>1.1175870895385742E-5</v>
+        <v>5.9232115745544434E-7</v>
       </c>
       <c r="J89" s="21"/>
       <c r="K89" s="21"/>
@@ -3830,37 +3835,37 @@
     </row>
     <row r="90" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A90" s="37" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B90" s="4">
-        <v>6</v>
+        <v>70</v>
       </c>
       <c r="C90" s="4">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D90" s="19">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>220</v>
       </c>
       <c r="E90" s="19">
-        <f>SUM(E48:E49)</f>
-        <v>106</v>
+        <f>SUM(E49:E55)</f>
+        <v>134</v>
       </c>
       <c r="F90" s="19">
         <f t="shared" si="1"/>
-        <v>636</v>
+        <v>29480</v>
       </c>
       <c r="G90" s="34">
         <f t="shared" si="2"/>
-        <v>0.62109375</v>
+        <v>28.7890625</v>
       </c>
       <c r="H90" s="34">
         <f t="shared" si="2"/>
-        <v>6.06536865234375E-4</v>
+        <v>2.811431884765625E-2</v>
       </c>
       <c r="I90" s="19">
         <f t="shared" si="2"/>
-        <v>5.9232115745544434E-7</v>
+        <v>2.7455389499664307E-5</v>
       </c>
       <c r="J90" s="21"/>
       <c r="K90" s="21"/>
@@ -3868,39 +3873,39 @@
       <c r="M90" s="20"/>
       <c r="N90" s="21"/>
     </row>
-    <row r="91" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:14" ht="23.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="37" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B91" s="4">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="C91" s="4">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D91" s="19">
         <f t="shared" si="0"/>
-        <v>220</v>
+        <v>70</v>
       </c>
       <c r="E91" s="19">
-        <f>SUM(E50:E56)</f>
-        <v>134</v>
+        <f>SUM(E57:E61)</f>
+        <v>16</v>
       </c>
       <c r="F91" s="19">
         <f t="shared" si="1"/>
-        <v>29480</v>
+        <v>1120</v>
       </c>
       <c r="G91" s="34">
         <f t="shared" si="2"/>
-        <v>28.7890625</v>
+        <v>1.09375</v>
       </c>
       <c r="H91" s="34">
         <f t="shared" si="2"/>
-        <v>2.811431884765625E-2</v>
+        <v>1.068115234375E-3</v>
       </c>
       <c r="I91" s="19">
         <f t="shared" si="2"/>
-        <v>2.7455389499664307E-5</v>
+        <v>1.0430812835693359E-6</v>
       </c>
       <c r="J91" s="21"/>
       <c r="K91" s="21"/>
@@ -3908,39 +3913,39 @@
       <c r="M91" s="20"/>
       <c r="N91" s="21"/>
     </row>
-    <row r="92" spans="1:14" ht="23.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="37" t="s">
-        <v>7</v>
-      </c>
-      <c r="B92" s="4">
-        <v>50</v>
-      </c>
-      <c r="C92" s="4">
-        <v>2</v>
+    <row r="92" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="A92" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="B92" s="18">
+        <v>250</v>
+      </c>
+      <c r="C92" s="18">
+        <v>25</v>
       </c>
       <c r="D92" s="19">
         <f t="shared" si="0"/>
-        <v>70</v>
+        <v>500</v>
       </c>
       <c r="E92" s="19">
-        <f>SUM(E58:E62)</f>
-        <v>16</v>
+        <f>SUM(E62:E65)</f>
+        <v>12</v>
       </c>
       <c r="F92" s="19">
         <f t="shared" si="1"/>
-        <v>1120</v>
+        <v>6000</v>
       </c>
       <c r="G92" s="34">
         <f t="shared" si="2"/>
-        <v>1.09375</v>
+        <v>5.859375</v>
       </c>
       <c r="H92" s="34">
         <f t="shared" si="2"/>
-        <v>1.068115234375E-3</v>
+        <v>5.7220458984375E-3</v>
       </c>
       <c r="I92" s="19">
         <f t="shared" si="2"/>
-        <v>1.0430812835693359E-6</v>
+        <v>5.5879354476928711E-6</v>
       </c>
       <c r="J92" s="21"/>
       <c r="K92" s="21"/>
@@ -3950,37 +3955,37 @@
     </row>
     <row r="93" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A93" s="35" t="s">
-        <v>8</v>
-      </c>
-      <c r="B93" s="18">
-        <v>250</v>
-      </c>
-      <c r="C93" s="18">
-        <v>25</v>
+        <v>9</v>
+      </c>
+      <c r="B93" s="38">
+        <v>30000000</v>
+      </c>
+      <c r="C93" s="38">
+        <v>33000000</v>
       </c>
       <c r="D93" s="19">
         <f t="shared" si="0"/>
-        <v>500</v>
+        <v>360000000</v>
       </c>
       <c r="E93" s="19">
-        <f>SUM(E63:E66)</f>
-        <v>12</v>
+        <f>SUM(E66:E69)</f>
+        <v>21</v>
       </c>
       <c r="F93" s="19">
         <f t="shared" si="1"/>
-        <v>6000</v>
+        <v>7560000000</v>
       </c>
       <c r="G93" s="34">
         <f t="shared" si="2"/>
-        <v>5.859375</v>
+        <v>7382812.5</v>
       </c>
       <c r="H93" s="34">
         <f t="shared" si="2"/>
-        <v>5.7220458984375E-3</v>
+        <v>7209.77783203125</v>
       </c>
       <c r="I93" s="19">
         <f t="shared" si="2"/>
-        <v>5.5879354476928711E-6</v>
+        <v>7.0407986640930176</v>
       </c>
       <c r="J93" s="21"/>
       <c r="K93" s="21"/>
@@ -3990,37 +3995,37 @@
     </row>
     <row r="94" spans="1:14" ht="15" x14ac:dyDescent="0.25">
       <c r="A94" s="35" t="s">
-        <v>9</v>
-      </c>
-      <c r="B94" s="38">
-        <v>30000000</v>
-      </c>
-      <c r="C94" s="38">
-        <v>33000000</v>
+        <v>10</v>
+      </c>
+      <c r="B94" s="18">
+        <v>30000</v>
+      </c>
+      <c r="C94" s="18">
+        <v>36000</v>
       </c>
       <c r="D94" s="19">
         <f t="shared" si="0"/>
-        <v>360000000</v>
+        <v>390000</v>
       </c>
       <c r="E94" s="19">
-        <f>SUM(E67:E70)</f>
+        <f>SUM(E70:E74)</f>
         <v>21</v>
       </c>
       <c r="F94" s="19">
         <f t="shared" si="1"/>
-        <v>7560000000</v>
+        <v>8190000</v>
       </c>
       <c r="G94" s="34">
         <f t="shared" si="2"/>
-        <v>7382812.5</v>
+        <v>7998.046875</v>
       </c>
       <c r="H94" s="34">
         <f t="shared" si="2"/>
-        <v>7209.77783203125</v>
+        <v>7.8105926513671875</v>
       </c>
       <c r="I94" s="19">
         <f t="shared" si="2"/>
-        <v>7.0407986640930176</v>
+        <v>7.627531886100769E-3</v>
       </c>
       <c r="J94" s="21"/>
       <c r="K94" s="21"/>
@@ -4029,38 +4034,38 @@
       <c r="N94" s="21"/>
     </row>
     <row r="95" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A95" s="35" t="s">
-        <v>10</v>
+      <c r="A95" s="23" t="s">
+        <v>22</v>
       </c>
       <c r="B95" s="18">
-        <v>30000</v>
+        <v>250</v>
       </c>
       <c r="C95" s="18">
-        <v>36000</v>
+        <v>39</v>
       </c>
       <c r="D95" s="19">
         <f t="shared" si="0"/>
-        <v>390000</v>
+        <v>640</v>
       </c>
       <c r="E95" s="19">
-        <f>SUM(E71:E75)</f>
-        <v>21</v>
+        <f>SUM(E75:E79)</f>
+        <v>135</v>
       </c>
       <c r="F95" s="19">
         <f t="shared" si="1"/>
-        <v>8190000</v>
+        <v>86400</v>
       </c>
       <c r="G95" s="34">
         <f t="shared" si="2"/>
-        <v>7998.046875</v>
+        <v>84.375</v>
       </c>
       <c r="H95" s="34">
         <f t="shared" si="2"/>
-        <v>7.8105926513671875</v>
+        <v>8.23974609375E-2</v>
       </c>
       <c r="I95" s="19">
         <f t="shared" si="2"/>
-        <v>7.627531886100769E-3</v>
+        <v>8.0466270446777344E-5</v>
       </c>
       <c r="J95" s="21"/>
       <c r="K95" s="21"/>
@@ -4069,39 +4074,14 @@
       <c r="N95" s="21"/>
     </row>
     <row r="96" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A96" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B96" s="18">
-        <v>250</v>
-      </c>
-      <c r="C96" s="18">
-        <v>39</v>
-      </c>
-      <c r="D96" s="19">
-        <f t="shared" si="0"/>
-        <v>640</v>
-      </c>
-      <c r="E96" s="19">
-        <f>SUM(E76:E80)</f>
-        <v>135</v>
-      </c>
-      <c r="F96" s="19">
-        <f t="shared" si="1"/>
-        <v>86400</v>
-      </c>
-      <c r="G96" s="34">
-        <f t="shared" si="2"/>
-        <v>84.375</v>
-      </c>
-      <c r="H96" s="34">
-        <f t="shared" si="2"/>
-        <v>8.23974609375E-2</v>
-      </c>
-      <c r="I96" s="19">
-        <f t="shared" si="2"/>
-        <v>8.0466270446777344E-5</v>
-      </c>
+      <c r="A96"/>
+      <c r="B96"/>
+      <c r="C96"/>
+      <c r="D96"/>
+      <c r="E96"/>
+      <c r="G96"/>
+      <c r="H96"/>
+      <c r="I96"/>
       <c r="J96" s="21"/>
       <c r="K96" s="21"/>
       <c r="L96" s="20"/>
@@ -4109,44 +4089,45 @@
       <c r="N96" s="21"/>
     </row>
     <row r="97" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A97"/>
-      <c r="B97"/>
-      <c r="C97"/>
-      <c r="D97"/>
-      <c r="E97"/>
-      <c r="G97"/>
-      <c r="H97"/>
-      <c r="I97"/>
+      <c r="A97" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="B97" s="40"/>
+      <c r="C97" s="40"/>
+      <c r="D97" s="21"/>
+      <c r="E97" s="21"/>
+      <c r="F97" s="19">
+        <f>SUM(F84:F95)</f>
+        <v>9608453436</v>
+      </c>
+      <c r="G97" s="19">
+        <f>SUM(G84:G95)</f>
+        <v>9383255.30859375</v>
+      </c>
+      <c r="H97" s="19">
+        <f>SUM(H84:H95)</f>
+        <v>9163.335262298584</v>
+      </c>
+      <c r="I97" s="19">
+        <f>SUM(I84:I95)</f>
+        <v>8.9485695920884609</v>
+      </c>
       <c r="J97" s="21"/>
       <c r="K97" s="21"/>
       <c r="L97" s="20"/>
       <c r="M97" s="20"/>
       <c r="N97" s="21"/>
     </row>
-    <row r="98" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A98" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="B98" s="40"/>
-      <c r="C98" s="40"/>
+    <row r="98" spans="1:14" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="21"/>
+      <c r="B98" s="21"/>
+      <c r="C98" s="21"/>
       <c r="D98" s="21"/>
       <c r="E98" s="21"/>
-      <c r="F98" s="19">
-        <f>SUM(F85:F96)</f>
-        <v>9608455686</v>
-      </c>
-      <c r="G98" s="19">
-        <f>SUM(G85:G96)</f>
-        <v>9383257.505859375</v>
-      </c>
-      <c r="H98" s="19">
-        <f>SUM(H85:H96)</f>
-        <v>9163.3374080657959</v>
-      </c>
-      <c r="I98" s="19">
-        <f>SUM(I85:I96)</f>
-        <v>8.9485716875642538</v>
-      </c>
+      <c r="F98" s="21"/>
+      <c r="G98" s="21"/>
+      <c r="H98" s="21"/>
+      <c r="I98" s="21"/>
       <c r="J98" s="21"/>
       <c r="K98" s="21"/>
       <c r="L98" s="20"/>
@@ -4154,47 +4135,47 @@
       <c r="N98" s="21"/>
     </row>
     <row r="99" spans="1:14" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="21"/>
-      <c r="B99" s="21"/>
-      <c r="C99" s="21"/>
-      <c r="D99" s="21"/>
+      <c r="A99" s="45" t="s">
+        <v>99</v>
+      </c>
+      <c r="B99" s="45"/>
+      <c r="C99" s="45"/>
+      <c r="D99" s="41">
+        <v>0.4</v>
+      </c>
       <c r="E99" s="21"/>
-      <c r="F99" s="21"/>
-      <c r="G99" s="21"/>
-      <c r="H99" s="21"/>
-      <c r="I99" s="21"/>
+      <c r="F99" s="19">
+        <f>F97*1.4</f>
+        <v>13451834810.4</v>
+      </c>
+      <c r="G99" s="19">
+        <f>G97*1.4</f>
+        <v>13136557.43203125</v>
+      </c>
+      <c r="H99" s="19">
+        <f>H97*1.4</f>
+        <v>12828.669367218017</v>
+      </c>
+      <c r="I99" s="19">
+        <f>I97*1.4</f>
+        <v>12.527997428923845</v>
+      </c>
       <c r="J99" s="21"/>
       <c r="K99" s="21"/>
       <c r="L99" s="20"/>
       <c r="M99" s="20"/>
       <c r="N99" s="21"/>
     </row>
-    <row r="100" spans="1:14" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="45" t="s">
-        <v>100</v>
-      </c>
-      <c r="B100" s="45"/>
-      <c r="C100" s="45"/>
-      <c r="D100" s="41">
-        <v>0.4</v>
-      </c>
+    <row r="100" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="A100" s="23"/>
+      <c r="B100" s="18"/>
+      <c r="C100" s="18"/>
+      <c r="D100" s="22"/>
       <c r="E100" s="21"/>
-      <c r="F100" s="19">
-        <f>F98*1.4</f>
-        <v>13451837960.4</v>
-      </c>
-      <c r="G100" s="19">
-        <f>G98*1.4</f>
-        <v>13136560.508203125</v>
-      </c>
-      <c r="H100" s="19">
-        <f>H98*1.4</f>
-        <v>12828.672371292114</v>
-      </c>
-      <c r="I100" s="19">
-        <f>I98*1.4</f>
-        <v>12.528000362589955</v>
-      </c>
+      <c r="F100" s="20"/>
+      <c r="G100" s="20"/>
+      <c r="H100" s="20"/>
+      <c r="I100" s="21"/>
       <c r="J100" s="21"/>
       <c r="K100" s="21"/>
       <c r="L100" s="20"/>
@@ -4234,15 +4215,6 @@
       <c r="N102" s="21"/>
     </row>
     <row r="103" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A103" s="23"/>
-      <c r="B103" s="18"/>
-      <c r="C103" s="18"/>
-      <c r="D103" s="22"/>
-      <c r="E103" s="21"/>
-      <c r="F103" s="20"/>
-      <c r="G103" s="20"/>
-      <c r="H103" s="20"/>
-      <c r="I103" s="21"/>
       <c r="J103" s="21"/>
       <c r="K103" s="21"/>
       <c r="L103" s="20"/>
@@ -4264,6 +4236,15 @@
       <c r="N105" s="21"/>
     </row>
     <row r="106" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="A106" s="23"/>
+      <c r="B106" s="18"/>
+      <c r="C106" s="18"/>
+      <c r="D106" s="22"/>
+      <c r="E106" s="21"/>
+      <c r="F106" s="20"/>
+      <c r="G106" s="20"/>
+      <c r="H106" s="20"/>
+      <c r="I106" s="21"/>
       <c r="J106" s="21"/>
       <c r="K106" s="21"/>
       <c r="L106" s="20"/>
@@ -4366,119 +4347,103 @@
       <c r="M112" s="20"/>
       <c r="N112" s="21"/>
     </row>
-    <row r="113" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="A113" s="23"/>
-      <c r="B113" s="18"/>
-      <c r="C113" s="18"/>
-      <c r="D113" s="22"/>
-      <c r="E113" s="21"/>
-      <c r="F113" s="20"/>
-      <c r="G113" s="20"/>
-      <c r="H113" s="20"/>
-      <c r="I113" s="21"/>
+    <row r="113" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J113" s="21"/>
       <c r="K113" s="21"/>
       <c r="L113" s="20"/>
       <c r="M113" s="20"/>
       <c r="N113" s="21"/>
     </row>
-    <row r="114" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="114" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J114" s="21"/>
       <c r="K114" s="21"/>
       <c r="L114" s="20"/>
       <c r="M114" s="20"/>
       <c r="N114" s="21"/>
     </row>
-    <row r="115" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="115" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J115" s="21"/>
       <c r="K115" s="21"/>
       <c r="L115" s="20"/>
       <c r="M115" s="20"/>
       <c r="N115" s="21"/>
     </row>
-    <row r="116" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="116" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J116" s="21"/>
       <c r="K116" s="21"/>
       <c r="L116" s="20"/>
       <c r="M116" s="20"/>
       <c r="N116" s="21"/>
     </row>
-    <row r="117" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="117" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J117" s="21"/>
       <c r="K117" s="21"/>
       <c r="L117" s="20"/>
       <c r="M117" s="20"/>
       <c r="N117" s="21"/>
     </row>
-    <row r="118" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="118" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J118" s="21"/>
       <c r="K118" s="21"/>
       <c r="L118" s="20"/>
       <c r="M118" s="20"/>
       <c r="N118" s="21"/>
     </row>
-    <row r="119" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="119" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J119" s="21"/>
       <c r="K119" s="21"/>
       <c r="L119" s="20"/>
       <c r="M119" s="20"/>
       <c r="N119" s="21"/>
     </row>
-    <row r="120" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="120" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J120" s="21"/>
       <c r="K120" s="21"/>
       <c r="L120" s="20"/>
       <c r="M120" s="20"/>
       <c r="N120" s="21"/>
     </row>
-    <row r="121" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="121" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J121" s="21"/>
       <c r="K121" s="21"/>
       <c r="L121" s="20"/>
       <c r="M121" s="20"/>
       <c r="N121" s="21"/>
     </row>
-    <row r="122" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="122" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J122" s="21"/>
       <c r="K122" s="21"/>
       <c r="L122" s="20"/>
       <c r="M122" s="20"/>
       <c r="N122" s="21"/>
     </row>
-    <row r="123" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="123" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J123" s="21"/>
       <c r="K123" s="21"/>
       <c r="L123" s="20"/>
       <c r="M123" s="20"/>
       <c r="N123" s="21"/>
     </row>
-    <row r="124" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="124" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J124" s="21"/>
       <c r="K124" s="21"/>
       <c r="L124" s="20"/>
       <c r="M124" s="20"/>
       <c r="N124" s="21"/>
     </row>
-    <row r="125" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="125" spans="10:14" ht="15" x14ac:dyDescent="0.25">
       <c r="J125" s="21"/>
       <c r="K125" s="21"/>
       <c r="L125" s="20"/>
       <c r="M125" s="20"/>
       <c r="N125" s="21"/>
     </row>
-    <row r="126" spans="1:14" ht="15" x14ac:dyDescent="0.25">
-      <c r="J126" s="21"/>
-      <c r="K126" s="21"/>
-      <c r="L126" s="20"/>
-      <c r="M126" s="20"/>
-      <c r="N126" s="21"/>
-    </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A81:B81"/>
-    <mergeCell ref="A82:F82"/>
-    <mergeCell ref="A83:B83"/>
-    <mergeCell ref="A100:C100"/>
+    <mergeCell ref="A80:B80"/>
+    <mergeCell ref="A81:F81"/>
+    <mergeCell ref="A82:B82"/>
+    <mergeCell ref="A99:C99"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Fix selection of rows in Speicherplatzberechnung
</commit_message>
<xml_diff>
--- a/Speicherplatzberechnung_Bäckereikette.xlsx
+++ b/Speicherplatzberechnung_Bäckereikette.xlsx
@@ -4127,24 +4127,24 @@
         <v>390000</v>
       </c>
       <c r="E95" s="17" t="n">
-        <f aca="false">SUM(E71:E75)</f>
-        <v>21</v>
+        <f aca="false">SUM(E70:E74)</f>
+        <v>20</v>
       </c>
       <c r="F95" s="17" t="n">
         <f aca="false">D95*E95</f>
-        <v>8190000</v>
+        <v>7800000</v>
       </c>
       <c r="G95" s="34" t="n">
         <f aca="false">F95/1024</f>
-        <v>7998.046875</v>
+        <v>7617.1875</v>
       </c>
       <c r="H95" s="34" t="n">
         <f aca="false">G95/1024</f>
-        <v>7.81059265136719</v>
+        <v>7.43865966796875</v>
       </c>
       <c r="I95" s="17" t="n">
         <f aca="false">H95/1024</f>
-        <v>0.00762753188610077</v>
+        <v>0.00726431608200073</v>
       </c>
       <c r="J95" s="19"/>
       <c r="K95" s="19"/>
@@ -4209,19 +4209,19 @@
       <c r="E98" s="19"/>
       <c r="F98" s="17" t="n">
         <f aca="false">SUM(F85:F96)</f>
-        <v>9608476476</v>
+        <v>9608086476</v>
       </c>
       <c r="G98" s="17" t="n">
         <f aca="false">SUM(G85:G96)</f>
-        <v>9383277.80859375</v>
+        <v>9382896.94921875</v>
       </c>
       <c r="H98" s="17" t="n">
         <f aca="false">SUM(H85:H96)</f>
-        <v>9163.35723495483</v>
+        <v>9162.98530197144</v>
       </c>
       <c r="I98" s="17" t="n">
         <f aca="false">SUM(I85:I96)</f>
-        <v>8.94859104976059</v>
+        <v>8.94822783395649</v>
       </c>
       <c r="J98" s="19"/>
       <c r="K98" s="19"/>
@@ -4259,19 +4259,19 @@
       <c r="E100" s="19"/>
       <c r="F100" s="17" t="n">
         <f aca="false">F98*1.4</f>
-        <v>13451867066.4</v>
+        <v>13451321066.4</v>
       </c>
       <c r="G100" s="17" t="n">
         <f aca="false">G98*1.4</f>
-        <v>13136588.9320313</v>
+        <v>13136055.7289063</v>
       </c>
       <c r="H100" s="17" t="n">
         <f aca="false">H98*1.4</f>
-        <v>12828.7001289368</v>
+        <v>12828.17942276</v>
       </c>
       <c r="I100" s="17" t="n">
         <f aca="false">I98*1.4</f>
-        <v>12.5280274696648</v>
+        <v>12.5275189675391</v>
       </c>
       <c r="J100" s="19"/>
       <c r="K100" s="19"/>

</xml_diff>